<commit_message>
Add automatic news parser and Docker setup
</commit_message>
<xml_diff>
--- a/database/book.xlsx
+++ b/database/book.xlsx
@@ -453,440 +453,440 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Уникальная выставка продолжает работу в Пушкинской библиотеке</t>
+          <t>Триста тысяч за храм без креста: Госдума усиливает штрафом защиту чувств верующих</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>21:31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Она посвящена монетам пушкинской эпохи</t>
+          <t>Изображение православного храма без креста грозит крупным штрафом</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182687</t>
+          <t>https://zab.ru/news/194074</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Почти 9 из 10 женщин в Забайкалье не курят</t>
+          <t>В Забайкалье за сутки горели почти 839 гектаров</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>13:11</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Статистикой поделились в Забайкалкрайстате</t>
+          <t>Забайкалье продолжает страдать от пожаров</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182680</t>
+          <t>https://zab.ru/news/194073</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Экстренное предупреждение снова объявлено в Забайкалье</t>
+          <t>В Забайкалье инспекторы ДПС остановили 61 пьяного водителя за прошедшие выходные</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Жителям региона рекомендуется проявлять осторожность</t>
+          <t>Пугающая статистика по ДТП и пьяным водителям</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182683</t>
+          <t>https://zab.ru/news/194072</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Соблюдаете ли вы режим питания?</t>
+          <t>Овечкин и отметка в 1000 голов НХЛ: что это говорит о снайперской игре в современном хоккее</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11:12</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Доступно пять вариантов ответа</t>
+          <t>Что это говорит о снайперской игре в современном хоккее</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182682</t>
+          <t>https://zab.ru/news/194071</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Влиятельность Осипова по-прежнему на низком уровне</t>
+          <t>Экс-главу Фонда развития Забайкалья Наталью Макарову задержали и доставили в Читу</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Он находится среди аутсайдеров</t>
+          <t>Официальной информации ещё нет</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182679</t>
+          <t>https://zab.ru/news/194070</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Восемь улиц краевого центра останутся сегодня без света</t>
+          <t>ЛДПР предложила отменить детские пособия для иностранных граждан</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09:08</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ожидаются плановые ремонтные работы</t>
+          <t>Леонид Слуцкий направил обращение вице-премьеру Татьяне Голиковой</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182678</t>
+          <t>https://zab.ru/news/194069</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Гороскоп для жителей Забайкальского края на 9 марта</t>
+          <t>В Забайкалье зафиксировано 39 случаев укусов клещей</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Звезды гороскопа не склоняют к тому, чтобы сидеть в четырех стенах</t>
+          <t>Также страдают дети</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182319</t>
+          <t>https://zab.ru/news/194068</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Большинству опрошенных женщин ничего не подарили</t>
+          <t>Автобусы №5 и №19 возобновят движение по прежней схеме с 13 апреля</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>22:41</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Грустные результаты опроса</t>
+          <t>Читинские автобусы ездят по старому маршруту</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182677</t>
+          <t>https://zab.ru/news/194066</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Снег и ветер обрушатся на Забайкалье</t>
+          <t>Рекламный рынок Читы под вопросом: решения принимал чиновник, уволенный за утрату доверия</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Прогноз погоды на 9 марта</t>
+          <t>Что станет с рекламным рынком после ухода Зудилова?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182676</t>
+          <t>https://zab.ru/news/194064</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>В Забайкалье начнут борьбу с алкоголем</t>
+          <t>Забайкалье попало в топ-5 по снижению потребления алкоголя</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Будет создана специальная комиссия</t>
+          <t>Общероссийская тенденция на трезвость</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182675</t>
+          <t>https://zab.ru/news/194063</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Забайкальцы нарубили дров на пять миллионов за неделю</t>
+          <t>ZAB.RU поздравляет с Пасхой</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>10:19</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Виновных будут искать</t>
+          <t>Христос воскресе! С праздником Пасхи всех православных!</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182674</t>
+          <t>https://zab.ru/news/194065</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Жители Забайкалья стали реже умирать от туберкулеза</t>
+          <t>Вратарь как первый пасующий: как голкипер стал частью билдапа</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>18:29</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Об этом говорят данные статистики</t>
+          <t>как голкипер стал частью билдапа</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182673</t>
+          <t>https://zab.ru/news/194067</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Забайкалец лишился свободы из-за неуплаты алиментов</t>
+          <t>Юрий Трутнев: регионы Дальнего Востока должны быть готовы к паводкам и пожарам 2026 года</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Он избегал наказания и снова попал под суд</t>
+          <t>На заседании совета ДФО обсудили подготовку регионов к прохождению паводкоопасного периода и пожароопасного сезона</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182672</t>
+          <t>https://zab.ru/news/194062</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>При ликвидации лесных пожаров впервые задействуют аэролодки</t>
+          <t>В Иркутской области 95 населенных пунктов рискуют попасть в зону паводка</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Пожары могут начаться уже в марте</t>
+          <t>Под угрозой подтопления из-за весеннего паводка оказались несколько населенных пунктов</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182671</t>
+          <t>https://zab.ru/news/194060</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>В МЧС предупредили об усилении ветра</t>
+          <t>В Бурятии мужчина задушил пожилого соседа после пьяной ссоры</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Порывы будут доходить до 20 м/с</t>
+          <t>Подробности преступления</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182670</t>
+          <t>https://zab.ru/news/194056</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Продукты стали дороже в Забайкалье</t>
+          <t>Петербургские депутаты решили разобраться с самокатами</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Цены выросли до 2,6%</t>
+          <t>Депутаты снова пытаются понять, что и как делать с электросамокатами</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182669</t>
+          <t>https://zab.ru/news/194055</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Спасатели дважды спасали запертых людей в Чите</t>
+          <t>Госдума удвоит список законных поводов для выдворения мигрантов</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Оба случая связаны с детьми</t>
+          <t>Предлагаемый законопроект увеличит количество «депортационных» статей вдвое</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182668</t>
+          <t>https://zab.ru/news/194054</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Жительница аварийного дома в Новой Чаре обратилась к Бастрыкину</t>
+          <t>В Забайкалье прокуратура направила в суд уголовное дело по обвинению начальника лесхоза в незаконной вырубке леса</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12:16</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Началась проверка</t>
+          <t>Юлия Макарова из «Забайкаллесхоза» организовала сплошную вырубку живого леса вместо санитарной</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182667</t>
+          <t>https://zab.ru/news/194053</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Бензин снова подорожал в Забайкалье</t>
+          <t>Адвокат из Читы отдал мошенникам 1,2 млн рублей из-за страха уголовки</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Топливо тоже стало дороже</t>
+          <t>Позвонили с почты, напугали госизменой — читинец оформил кредиты сам</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182665</t>
+          <t>https://zab.ru/news/194052</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Опрос для женщин: что вам подарили?</t>
+          <t>Как скаутинг перешёл от хайлайтов к данным: почему трансферный рынок больше не ищет звёзд</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Он действителен до конца дня</t>
+          <t>Почему трансферный рынок больше не ищет звёзд?</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://zab.ru/news/182664</t>
+          <t>https://zab.ru/news/194059</t>
         </is>
       </c>
     </row>

</xml_diff>